<commit_message>
Fix: Textbook management refactor and mojibake
</commit_message>
<xml_diff>
--- a/apps/admin/public/textbook_summary_template.xlsx
+++ b/apps/admin/public/textbook_summary_template.xlsx
@@ -3,13 +3,16 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84895970-EC4F-49C4-90C5-C989C160A439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E62902C-70C9-47CC-84A2-284F8D7FB327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$B$2</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -28,23 +31,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
-  <si>
-    <t>注文日時</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>教科</t>
   </si>
   <si>
-    <t>高校名</t>
-  </si>
-  <si>
-    <t>ご担当者名</t>
-  </si>
-  <si>
-    <t>メールアドレス</t>
-  </si>
-  <si>
     <t>学校TEL</t>
   </si>
   <si>
@@ -54,13 +45,7 @@
     <t>教材名</t>
   </si>
   <si>
-    <t>出版社</t>
-  </si>
-  <si>
     <t>本体価格</t>
-  </si>
-  <si>
-    <t>対象学年</t>
   </si>
   <si>
     <t>生徒用数</t>
@@ -110,10 +95,42 @@
     <phoneticPr fontId="3"/>
   </si>
   <si>
-    <t>合計冊数</t>
-    <rPh sb="0" eb="4">
-      <t>ゴウケイサツスウ</t>
+    <t>注文日</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>帳合</t>
+    <rPh sb="0" eb="2">
+      <t>チョウアイ</t>
     </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>出版社</t>
+    <rPh sb="0" eb="3">
+      <t>シュッパンシャ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>学校名</t>
+    <rPh sb="0" eb="1">
+      <t>ガク</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>担当先生</t>
+    <rPh sb="0" eb="2">
+      <t>タントウ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>センセイ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>学年</t>
     <phoneticPr fontId="3"/>
   </si>
 </sst>
@@ -547,104 +564,98 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y2"/>
+  <dimension ref="A1:X2"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="10" max="12" width="9" style="3"/>
+    <col min="11" max="13" width="9" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="P1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="T1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>21</v>
-      </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.15">
-      <c r="K2" s="3">
-        <f>J2*1.1</f>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.15">
+      <c r="L2" s="3">
+        <f>K2*1.1</f>
         <v>0</v>
       </c>
-      <c r="L2" s="3">
-        <f>K2*P2</f>
-        <v>0</v>
-      </c>
-      <c r="P2">
-        <f>N2+O2</f>
+      <c r="M2" s="3">
+        <f>L2*I2</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="B1:B2" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>